<commit_message>
Deploy: Commission report enhancements + server deployment
- Added Group By toggle (Client/Individual) to Quarterly Commission report
- Fixed Excel export for both grouping modes
- Added 'Include commission lines with no payment' checkbox
- Added deploy.sh for Python/FastAPI server deployment via PM2
- Added sqlalchemy, psycopg2-binary, python-multipart to requirements.txt
- Updated backend commission API with include_no_payment parameter
</commit_message>
<xml_diff>
--- a/Payroll/Vijay Payroll.xlsx
+++ b/Payroll/Vijay Payroll.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/matthewmohebbi/Documents/AntiGravity-SAP report/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/matthewmohebbi/Documents/AntiGravity-SAP report/Payroll/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2449ED6-370A-5646-AD0F-8531698B6262}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E97D7F21-BBE0-A94D-BDC5-2A0A6EFD9E9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{3E3A6D6E-9638-4FA2-AEF6-DCF30D5B383C}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="36320" windowHeight="18980" xr2:uid="{3E3A6D6E-9638-4FA2-AEF6-DCF30D5B383C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -262,9 +262,6 @@
     <t xml:space="preserve">401K Loan </t>
   </si>
   <si>
-    <t>CHILD SUPPORT + CHILD SUPPORT 1+ CHILD SUPPORT 2</t>
-  </si>
-  <si>
     <t xml:space="preserve">DENTAL + HUMANA DENTAL </t>
   </si>
   <si>
@@ -364,9 +361,6 @@
     <t>EMPLOYER LIABILITIES Total</t>
   </si>
   <si>
-    <t>1100 MISC PAY</t>
-  </si>
-  <si>
     <t>ADVANCE PAYMENT</t>
   </si>
   <si>
@@ -383,6 +377,12 @@
   </si>
   <si>
     <t>RE-TRAINING + TRAINING  + TRAININGOT HOURS</t>
+  </si>
+  <si>
+    <t>CHILD SUPPORT + CHILD SUPPORT1+ CHILD SUPPORT2+CHILD SUPPORT2 (2)+CHILD SUPPORT3</t>
+  </si>
+  <si>
+    <t>1099 MISC COMP +NET REIMBURSEM ENT +NET REIMBURSEM ENT</t>
   </si>
 </sst>
 </file>
@@ -908,13 +908,13 @@
         <v>53</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G1" s="5" t="s">
         <v>70</v>
@@ -931,7 +931,7 @@
         <v>54</v>
       </c>
       <c r="D2" s="10" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="F2" s="6"/>
       <c r="G2" s="10"/>
@@ -1005,7 +1005,7 @@
         <v>8</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C7" s="10" t="s">
         <v>54</v>
@@ -1021,7 +1021,7 @@
         <v>11</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C8" s="10" t="s">
         <v>54</v>
@@ -1060,7 +1060,7 @@
         <v>54</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F10" s="18"/>
       <c r="G10" s="10"/>
@@ -1248,7 +1248,7 @@
         <v>68</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C23" s="9" t="s">
         <v>67</v>
@@ -1326,7 +1326,7 @@
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A28" s="10" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B28" s="10" t="s">
         <v>64</v>
@@ -1400,8 +1400,8 @@
       <c r="B33" t="s">
         <v>35</v>
       </c>
-      <c r="D33" t="s">
-        <v>109</v>
+      <c r="D33" s="10" t="s">
+        <v>115</v>
       </c>
       <c r="F33" s="6"/>
       <c r="G33" s="10"/>
@@ -1411,10 +1411,10 @@
         <v>31</v>
       </c>
       <c r="B34" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D34" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F34" s="6"/>
       <c r="G34" s="6"/>
@@ -1423,7 +1423,7 @@
     </row>
     <row r="35" spans="1:10" s="20" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A35" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B35" s="19"/>
       <c r="C35" s="19"/>
@@ -1439,20 +1439,20 @@
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B36" t="s">
         <v>71</v>
       </c>
       <c r="E36" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="F36"/>
       <c r="G36" s="8"/>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B37" t="s">
         <v>72</v>
@@ -1471,20 +1471,20 @@
         <v>44</v>
       </c>
       <c r="E38" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="F38"/>
       <c r="G38" s="8"/>
     </row>
     <row r="39" spans="1:10" ht="48" x14ac:dyDescent="0.2">
       <c r="A39" s="16" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B39" t="s">
         <v>73</v>
       </c>
       <c r="E39" s="17" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="F39"/>
       <c r="G39" s="8"/>
@@ -1494,10 +1494,10 @@
         <v>46</v>
       </c>
       <c r="B40" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E40" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="F40"/>
       <c r="G40" s="8"/>
@@ -1510,33 +1510,33 @@
         <v>40</v>
       </c>
       <c r="E41" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F41"/>
       <c r="G41" s="8"/>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B42" t="s">
         <v>37</v>
       </c>
       <c r="E42" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="F42"/>
       <c r="G42" s="8"/>
     </row>
     <row r="43" spans="1:10" ht="48" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
+        <v>102</v>
+      </c>
+      <c r="B43" t="s">
         <v>103</v>
       </c>
-      <c r="B43" t="s">
-        <v>104</v>
-      </c>
       <c r="E43" s="17" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="F43"/>
       <c r="G43" s="8"/>
@@ -1549,20 +1549,20 @@
         <v>39</v>
       </c>
       <c r="E44" s="17" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F44"/>
       <c r="G44" s="8"/>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B45" t="s">
         <v>38</v>
       </c>
       <c r="E45" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F45"/>
       <c r="G45" s="8"/>
@@ -1575,7 +1575,7 @@
         <v>36</v>
       </c>
       <c r="E46" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F46"/>
       <c r="G46" s="8"/>
@@ -1585,10 +1585,10 @@
         <v>51</v>
       </c>
       <c r="B47" t="s">
+        <v>76</v>
+      </c>
+      <c r="E47" t="s">
         <v>77</v>
-      </c>
-      <c r="E47" t="s">
-        <v>78</v>
       </c>
       <c r="F47"/>
       <c r="G47" s="8"/>
@@ -1601,7 +1601,7 @@
         <v>41</v>
       </c>
       <c r="E49" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F49"/>
       <c r="G49" s="8"/>
@@ -1614,7 +1614,7 @@
         <v>43</v>
       </c>
       <c r="E50" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="F50"/>
       <c r="G50" s="8"/>
@@ -1627,7 +1627,7 @@
         <v>42</v>
       </c>
       <c r="E51" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F51"/>
       <c r="G51" s="8"/>
@@ -1640,14 +1640,14 @@
         <v>30</v>
       </c>
       <c r="E52" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F52"/>
       <c r="G52" s="8"/>
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A53" s="7" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B53" s="7"/>
       <c r="C53" s="7"/>
@@ -1667,12 +1667,12 @@
         <v>52</v>
       </c>
       <c r="B54" s="10" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C54" s="10"/>
       <c r="D54" s="10"/>
       <c r="E54" s="10" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F54" s="10"/>
       <c r="G54" s="6"/>
@@ -1684,12 +1684,12 @@
         <v>52</v>
       </c>
       <c r="B55" s="10" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C55" s="10"/>
       <c r="D55" s="10"/>
       <c r="E55" s="10" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F55" s="10"/>
       <c r="H55" s="14"/>
@@ -1697,7 +1697,7 @@
     </row>
     <row r="56" spans="1:10" s="20" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A56" s="19" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F56" s="21"/>
       <c r="G56" s="21"/>

</xml_diff>